<commit_message>
Updated Payment Method IDs for AdvIVRStoredPM TEst Case
</commit_message>
<xml_diff>
--- a/AdvIVRStoredPM.xlsx
+++ b/AdvIVRStoredPM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SoapData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0A2B1B-4DEF-4C1B-B42B-A33D2CCD179A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4065990-8D0B-452F-B3C8-1F8484765094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31406" yWindow="1123" windowWidth="28140" windowHeight="11803" activeTab="2" xr2:uid="{85B41B3E-B5F3-4D86-B0EB-E4C43EA08BD6}"/>
+    <workbookView xWindow="5362" yWindow="2858" windowWidth="21601" windowHeight="11324" firstSheet="2" activeTab="4" xr2:uid="{85B41B3E-B5F3-4D86-B0EB-E4C43EA08BD6}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateCCStoredPM" sheetId="1" r:id="rId1"/>
@@ -589,45 +589,24 @@
     <t>123000103</t>
   </si>
   <si>
-    <t>83197</t>
-  </si>
-  <si>
     <t>123000104</t>
   </si>
   <si>
-    <t>83198</t>
-  </si>
-  <si>
     <t>123000105</t>
   </si>
   <si>
-    <t>83199</t>
-  </si>
-  <si>
     <t>123000106</t>
   </si>
   <si>
-    <t>83200</t>
-  </si>
-  <si>
     <t>123000107</t>
   </si>
   <si>
-    <t>83201</t>
-  </si>
-  <si>
     <t>123000108</t>
   </si>
   <si>
-    <t>83202</t>
-  </si>
-  <si>
     <t>1230001102</t>
   </si>
   <si>
-    <t>83206</t>
-  </si>
-  <si>
     <t>PAL1</t>
   </si>
   <si>
@@ -847,12 +826,6 @@
     <t>1235511178</t>
   </si>
   <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>122025</t>
-  </si>
-  <si>
     <t>2028</t>
   </si>
   <si>
@@ -863,6 +836,33 @@
   </si>
   <si>
     <t>9006</t>
+  </si>
+  <si>
+    <t>122029</t>
+  </si>
+  <si>
+    <t>2029</t>
+  </si>
+  <si>
+    <t>114271</t>
+  </si>
+  <si>
+    <t>114272</t>
+  </si>
+  <si>
+    <t>114285</t>
+  </si>
+  <si>
+    <t>114286</t>
+  </si>
+  <si>
+    <t>114287</t>
+  </si>
+  <si>
+    <t>114288</t>
+  </si>
+  <si>
+    <t>114289</t>
   </si>
 </sst>
 </file>
@@ -1241,40 +1241,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22F9AEF9-6503-40FE-8219-A319EFB418E3}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.86328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.3984375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.3984375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="11.1328125" style="1" customWidth="1"/>
     <col min="17" max="17" width="17" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="9.140625" style="1"/>
+    <col min="18" max="18" width="6.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>69</v>
       </c>
@@ -1377,13 +1377,13 @@
         <v>20</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>24</v>
@@ -1440,7 +1440,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>70</v>
       </c>
@@ -1457,13 +1457,13 @@
         <v>33</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>24</v>
@@ -1520,7 +1520,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>71</v>
       </c>
@@ -1537,13 +1537,13 @@
         <v>34</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>24</v>
@@ -1600,7 +1600,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>72</v>
       </c>
@@ -1617,13 +1617,13 @@
         <v>35</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>24</v>
@@ -1680,7 +1680,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>73</v>
       </c>
@@ -1697,13 +1697,13 @@
         <v>67</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>24</v>
@@ -1760,7 +1760,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>74</v>
       </c>
@@ -1777,13 +1777,13 @@
         <v>54</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>24</v>
@@ -1840,7 +1840,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>75</v>
       </c>
@@ -1857,13 +1857,13 @@
         <v>20</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>24</v>
@@ -1908,7 +1908,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>76</v>
       </c>
@@ -1925,13 +1925,13 @@
         <v>33</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>24</v>
@@ -1976,7 +1976,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>77</v>
       </c>
@@ -1993,13 +1993,13 @@
         <v>34</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>24</v>
@@ -2044,7 +2044,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>78</v>
       </c>
@@ -2061,13 +2061,13 @@
         <v>35</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>24</v>
@@ -2112,7 +2112,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>59</v>
       </c>
@@ -2129,13 +2129,13 @@
         <v>20</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>24</v>
@@ -2192,7 +2192,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>61</v>
       </c>
@@ -2209,13 +2209,13 @@
         <v>20</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>24</v>
@@ -2272,7 +2272,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>63</v>
       </c>
@@ -2289,13 +2289,13 @@
         <v>20</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>24</v>
@@ -2352,7 +2352,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -2369,13 +2369,13 @@
         <v>20</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>24</v>
@@ -2445,40 +2445,40 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D4D5C8-6F34-4AE2-8796-F82A0BB3B401}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultColWidth="19.28515625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="19.265625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.3984375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.59765625" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="19.28515625" style="1"/>
+    <col min="18" max="18" width="6.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="19.265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>75</v>
       </c>
@@ -2581,13 +2581,13 @@
         <v>20</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>79</v>
@@ -2632,7 +2632,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>76</v>
       </c>
@@ -2649,13 +2649,13 @@
         <v>33</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>79</v>
@@ -2700,7 +2700,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>77</v>
       </c>
@@ -2717,13 +2717,13 @@
         <v>34</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>79</v>
@@ -2768,7 +2768,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>78</v>
       </c>
@@ -2785,13 +2785,13 @@
         <v>35</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>79</v>
@@ -2848,31 +2848,31 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D71CA8C4-34F9-4667-883D-8C9AB3ADB60A}">
   <dimension ref="A1:T21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="10.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.86328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.265625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="10.3984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1"/>
-    <col min="11" max="11" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1328125" style="1"/>
+    <col min="11" max="11" width="6.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.86328125" style="1" customWidth="1"/>
     <col min="17" max="17" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.85546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="13.5703125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="11.86328125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="13.59765625" style="1" customWidth="1"/>
     <col min="20" max="20" width="46" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="21" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>81</v>
       </c>
@@ -2951,13 +2951,13 @@
         <v>20</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>24</v>
@@ -2993,7 +2993,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>82</v>
       </c>
@@ -3010,13 +3010,13 @@
         <v>20</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>24</v>
@@ -3052,7 +3052,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
@@ -3069,13 +3069,13 @@
         <v>20</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>24</v>
@@ -3111,7 +3111,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>85</v>
       </c>
@@ -3131,13 +3131,13 @@
         <v>20</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>24</v>
@@ -3173,7 +3173,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>85</v>
       </c>
@@ -3193,13 +3193,13 @@
         <v>20</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>24</v>
@@ -3235,7 +3235,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>86</v>
       </c>
@@ -3252,13 +3252,13 @@
         <v>20</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>24</v>
@@ -3294,7 +3294,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>87</v>
       </c>
@@ -3311,13 +3311,13 @@
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>24</v>
@@ -3353,7 +3353,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>88</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>22</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>24</v>
@@ -3406,13 +3406,13 @@
         <v>47</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>89</v>
       </c>
@@ -3432,10 +3432,10 @@
         <v>20</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>24</v>
@@ -3471,7 +3471,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>90</v>
       </c>
@@ -3491,7 +3491,7 @@
         <v>20</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>22</v>
@@ -3530,7 +3530,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>91</v>
       </c>
@@ -3550,13 +3550,13 @@
         <v>20</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>25</v>
@@ -3589,7 +3589,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>92</v>
       </c>
@@ -3609,13 +3609,13 @@
         <v>20</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>24</v>
@@ -3648,7 +3648,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>93</v>
       </c>
@@ -3668,13 +3668,13 @@
         <v>20</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>24</v>
@@ -3707,7 +3707,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>94</v>
       </c>
@@ -3727,13 +3727,13 @@
         <v>20</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>24</v>
@@ -3766,7 +3766,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>95</v>
       </c>
@@ -3786,13 +3786,13 @@
         <v>20</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>24</v>
@@ -3828,7 +3828,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>96</v>
       </c>
@@ -3848,13 +3848,13 @@
         <v>20</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>24</v>
@@ -3890,7 +3890,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>97</v>
       </c>
@@ -3910,13 +3910,13 @@
         <v>20</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>24</v>
@@ -3952,7 +3952,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>98</v>
       </c>
@@ -3972,13 +3972,13 @@
         <v>106</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>24</v>
@@ -4014,7 +4014,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>99</v>
       </c>
@@ -4034,13 +4034,13 @@
         <v>107</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>24</v>
@@ -4076,7 +4076,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>100</v>
       </c>
@@ -4096,13 +4096,13 @@
         <v>108</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>22</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>24</v>
@@ -4151,48 +4151,48 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B82BD2A-CDCE-4C7C-8D4D-7376F79FC13B}">
   <dimension ref="A1:BH15"/>
-  <sheetFormatPr defaultColWidth="13.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="13.265625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="28.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.3984375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.3984375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="11.1328125" style="1" customWidth="1"/>
     <col min="17" max="17" width="17" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.28515625" style="1"/>
-    <col min="30" max="30" width="23.5703125" style="1" customWidth="1"/>
-    <col min="31" max="33" width="13.28515625" style="1"/>
-    <col min="34" max="34" width="16.42578125" style="1" customWidth="1"/>
-    <col min="35" max="52" width="13.28515625" style="1"/>
-    <col min="53" max="53" width="16.7109375" style="1" customWidth="1"/>
-    <col min="54" max="55" width="13.28515625" style="1"/>
-    <col min="56" max="56" width="21.7109375" style="1" customWidth="1"/>
-    <col min="57" max="16384" width="13.28515625" style="1"/>
+    <col min="18" max="18" width="6.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.265625" style="1"/>
+    <col min="30" max="30" width="23.59765625" style="1" customWidth="1"/>
+    <col min="31" max="33" width="13.265625" style="1"/>
+    <col min="34" max="34" width="16.3984375" style="1" customWidth="1"/>
+    <col min="35" max="52" width="13.265625" style="1"/>
+    <col min="53" max="53" width="16.73046875" style="1" customWidth="1"/>
+    <col min="54" max="55" width="13.265625" style="1"/>
+    <col min="56" max="56" width="21.73046875" style="1" customWidth="1"/>
+    <col min="57" max="16384" width="13.265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>125</v>
       </c>
@@ -4374,7 +4374,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>158</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>158</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>158</v>
       </c>
@@ -4866,7 +4866,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>158</v>
       </c>
@@ -5030,7 +5030,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>158</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>158</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>158</v>
       </c>
@@ -5510,7 +5510,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>158</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>158</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>158</v>
       </c>
@@ -5966,7 +5966,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>158</v>
       </c>
@@ -6130,7 +6130,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>158</v>
       </c>
@@ -6294,7 +6294,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="14" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>158</v>
       </c>
@@ -6458,7 +6458,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="15" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:60" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>158</v>
       </c>
@@ -6634,21 +6634,21 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7815927-229B-420D-B556-6514A6C920D3}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="62.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="1"/>
+    <col min="1" max="1" width="62.73046875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.265625" style="1"/>
     <col min="3" max="3" width="30" style="1" customWidth="1"/>
-    <col min="4" max="6" width="13.28515625" style="1"/>
-    <col min="7" max="7" width="16.42578125" style="1" customWidth="1"/>
-    <col min="8" max="25" width="13.28515625" style="1"/>
-    <col min="26" max="26" width="16.7109375" style="1" customWidth="1"/>
-    <col min="27" max="28" width="13.28515625" style="1"/>
-    <col min="29" max="29" width="21.7109375" style="1" customWidth="1"/>
-    <col min="30" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="6" width="13.265625" style="1"/>
+    <col min="7" max="7" width="16.3984375" style="1" customWidth="1"/>
+    <col min="8" max="25" width="13.265625" style="1"/>
+    <col min="26" max="26" width="16.73046875" style="1" customWidth="1"/>
+    <col min="27" max="28" width="13.265625" style="1"/>
+    <col min="29" max="29" width="21.73046875" style="1" customWidth="1"/>
+    <col min="30" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>125</v>
       </c>
@@ -6722,36 +6722,36 @@
         <v>181</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="AF1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="AA1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>131</v>
@@ -6814,7 +6814,7 @@
         <v>182</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>183</v>
+        <v>268</v>
       </c>
       <c r="Y2" s="1" t="s">
         <v>150</v>
@@ -6835,18 +6835,18 @@
         <v>154</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF2" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>131</v>
@@ -6906,10 +6906,10 @@
         <v>149</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>185</v>
+        <v>269</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>150</v>
@@ -6930,18 +6930,18 @@
         <v>154</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF3" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG3" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>131</v>
@@ -7001,10 +7001,10 @@
         <v>149</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>187</v>
+        <v>270</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>150</v>
@@ -7025,18 +7025,18 @@
         <v>154</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF4" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG4" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>131</v>
@@ -7096,10 +7096,10 @@
         <v>149</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>189</v>
+        <v>271</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>150</v>
@@ -7120,18 +7120,18 @@
         <v>154</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF5" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>131</v>
@@ -7191,10 +7191,10 @@
         <v>149</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>191</v>
+        <v>272</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>150</v>
@@ -7215,18 +7215,18 @@
         <v>154</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF6" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG6" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>131</v>
@@ -7286,10 +7286,10 @@
         <v>149</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>193</v>
+        <v>273</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>150</v>
@@ -7310,18 +7310,18 @@
         <v>154</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF7" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG7" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>131</v>
@@ -7381,10 +7381,10 @@
         <v>149</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>195</v>
+        <v>274</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>150</v>
@@ -7405,18 +7405,18 @@
         <v>154</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="AF8" s="1" t="s">
         <v>156</v>
       </c>
       <c r="AG8" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>131</v>
@@ -7446,12 +7446,12 @@
         <v>182</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>183</v>
+        <v>268</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>131</v>
@@ -7478,15 +7478,15 @@
         <v>139</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>185</v>
+        <v>269</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>131</v>
@@ -7513,15 +7513,15 @@
         <v>139</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>187</v>
+        <v>270</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>131</v>
@@ -7548,15 +7548,15 @@
         <v>139</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="X12" s="1" t="s">
-        <v>189</v>
+        <v>271</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>131</v>
@@ -7583,15 +7583,15 @@
         <v>139</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="X13" s="1" t="s">
-        <v>191</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>131</v>
@@ -7618,15 +7618,15 @@
         <v>139</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="X14" s="1" t="s">
-        <v>193</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>131</v>
@@ -7653,15 +7653,16 @@
         <v>139</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="X15" s="1" t="s">
-        <v>195</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -7671,12 +7672,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6024C524-EAFE-41AA-B57C-DE469EA75E7A}">
   <dimension ref="A1:AC5"/>
-  <sheetFormatPr defaultColWidth="31" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="31" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="16384" width="31" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>125</v>
       </c>
@@ -7687,96 +7688,96 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>251</v>
-      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>32</v>
@@ -7785,16 +7786,16 @@
         <v>53</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>49</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>48</v>
@@ -7803,7 +7804,7 @@
         <v>52</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>51</v>
@@ -7812,88 +7813,88 @@
         <v>45</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>46</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="Z2" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="W2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>268</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>44</v>

</xml_diff>